<commit_message>
xml finalizado faltando validação
</commit_message>
<xml_diff>
--- a/TemplateAC_YINSON.xlsx
+++ b/TemplateAC_YINSON.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-3150" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Template Formulário" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Formulário" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Template Formulário'!$A$1:$J$42</definedName>
@@ -456,7 +456,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -474,26 +474,26 @@
       <nvPicPr>
         <cNvPr id="2" name="Picture 1"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:srcRect l="7748" r="8481"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" l="7748" r="8481"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="149225" y="111125"/>
           <a:ext cx="1412875" cy="676151"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -518,26 +518,26 @@
       <nvPicPr>
         <cNvPr id="3" name="Picture 1"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:srcRect t="4047" b="4047"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" t="4047" b="4047"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="8131176" y="111125"/>
           <a:ext cx="1143000" cy="739644"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -868,7 +868,7 @@
       <c r="B2" s="13" t="n"/>
       <c r="C2" s="25" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Sensores de Temperatura</t>
+          <t>Análise Crítica de Calibração dos Transmissores de Pressão</t>
         </is>
       </c>
       <c r="D2" s="21" t="n"/>
@@ -928,7 +928,7 @@
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>27TT2502</t>
+          <t>28PT3507</t>
         </is>
       </c>
       <c r="G7" s="27" t="n"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>26-ODS-95 - TEM - 039</t>
+          <t>26-ODS-95 - PRE - 015</t>
         </is>
       </c>
       <c r="G8" s="27" t="n"/>
@@ -969,7 +969,7 @@
       </c>
       <c r="C9" s="35" t="inlineStr">
         <is>
-          <t>04/02/2026</t>
+          <t>29/01/2026</t>
         </is>
       </c>
       <c r="D9" s="28" t="n"/>
@@ -1493,7 +1493,7 @@
       <c r="G40" s="18" t="n"/>
       <c r="H40" s="19" t="inlineStr">
         <is>
-          <t>09/02/2026</t>
+          <t>02/02/2026</t>
         </is>
       </c>
       <c r="I40" s="20" t="n"/>
@@ -1525,9 +1525,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
-    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="C9:D9"/>
+    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B29:F29"/>

</xml_diff>

<commit_message>
ajuste AC Yinson FPSO - ATLANTA / tirada a geração de xml petro até que seja validada
</commit_message>
<xml_diff>
--- a/TemplateAC_YINSON.xlsx
+++ b/TemplateAC_YINSON.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-3150" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="13320" yWindow="-16485" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Formulário" sheetId="1" state="visible" r:id="rId1"/>
@@ -329,6 +329,10 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
@@ -337,8 +341,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -351,33 +373,11 @@
     <xf numFmtId="14" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -488,50 +488,6 @@
         <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="149225" y="111125"/>
           <a:ext cx="1412875" cy="676151"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>6</col>
-      <colOff>549276</colOff>
-      <row>0</row>
-      <rowOff>111125</rowOff>
-    </from>
-    <to>
-      <col>9</col>
-      <colOff>1</colOff>
-      <row>3</row>
-      <rowOff>50669</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Picture 1"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" t="4047" b="4047"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="8131176" y="111125"/>
-          <a:ext cx="1143000" cy="739644"/>
         </a:xfrm>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
@@ -852,16 +808,16 @@
   <dimension ref="B2:J41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1796875" defaultRowHeight="12"/>
   <cols>
-    <col width="1.26953125" customWidth="1" style="44" min="1" max="1"/>
-    <col width="23" customWidth="1" style="44" min="2" max="2"/>
-    <col width="22" customWidth="1" style="44" min="3" max="3"/>
-    <col width="18.453125" customWidth="1" style="44" min="4" max="4"/>
-    <col width="23.453125" bestFit="1" customWidth="1" style="44" min="5" max="5"/>
-    <col width="20.453125" customWidth="1" style="44" min="6" max="6"/>
-    <col width="8.1796875" customWidth="1" style="44" min="7" max="7"/>
-    <col width="8" customWidth="1" style="44" min="8" max="9"/>
-    <col width="9.1796875" customWidth="1" style="44" min="10" max="24"/>
-    <col width="9.1796875" customWidth="1" style="44" min="25" max="16384"/>
+    <col width="1.26953125" customWidth="1" style="27" min="1" max="1"/>
+    <col width="23" customWidth="1" style="27" min="2" max="2"/>
+    <col width="22" customWidth="1" style="27" min="3" max="3"/>
+    <col width="18.453125" customWidth="1" style="27" min="4" max="4"/>
+    <col width="23.453125" bestFit="1" customWidth="1" style="27" min="5" max="5"/>
+    <col width="20.453125" customWidth="1" style="27" min="6" max="6"/>
+    <col width="8.1796875" customWidth="1" style="27" min="7" max="7"/>
+    <col width="8" customWidth="1" style="27" min="8" max="9"/>
+    <col width="9.1796875" customWidth="1" style="27" min="10" max="25"/>
+    <col width="9.1796875" customWidth="1" style="27" min="26" max="16384"/>
   </cols>
   <sheetData>
     <row r="2" ht="37.5" customHeight="1">
@@ -906,7 +862,7 @@
       <c r="I5" s="14" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="43" t="n"/>
+      <c r="B6" s="26" t="n"/>
       <c r="J6" s="3" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -915,25 +871,25 @@
           <t>Cliente:</t>
         </is>
       </c>
-      <c r="C7" s="41" t="inlineStr">
+      <c r="C7" s="37" t="inlineStr">
         <is>
           <t>YINSON</t>
         </is>
       </c>
-      <c r="D7" s="28" t="n"/>
+      <c r="D7" s="30" t="n"/>
       <c r="E7" s="17" t="inlineStr">
         <is>
           <t>TAG do instrumento:</t>
         </is>
       </c>
-      <c r="F7" s="26" t="inlineStr">
-        <is>
-          <t>28PT3507</t>
-        </is>
-      </c>
-      <c r="G7" s="27" t="n"/>
-      <c r="H7" s="27" t="n"/>
-      <c r="I7" s="28" t="n"/>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>27PT2001</t>
+        </is>
+      </c>
+      <c r="G7" s="29" t="n"/>
+      <c r="H7" s="29" t="n"/>
+      <c r="I7" s="30" t="n"/>
     </row>
     <row r="8" ht="14.5" customHeight="1">
       <c r="B8" s="17" t="inlineStr">
@@ -941,25 +897,25 @@
           <t>Localização:</t>
         </is>
       </c>
-      <c r="C8" s="40" t="inlineStr">
+      <c r="C8" s="36" t="inlineStr">
         <is>
           <t>FPSO Maria Quitéria</t>
         </is>
       </c>
-      <c r="D8" s="28" t="n"/>
+      <c r="D8" s="30" t="n"/>
       <c r="E8" s="17" t="inlineStr">
         <is>
           <t>Número do Certificado:</t>
         </is>
       </c>
-      <c r="F8" s="26" t="inlineStr">
-        <is>
-          <t>26-ODS-95 - PRE - 015</t>
-        </is>
-      </c>
-      <c r="G8" s="27" t="n"/>
-      <c r="H8" s="27" t="n"/>
-      <c r="I8" s="28" t="n"/>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>24‐ODS‐95 ‐ PRE ‐ 974</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="n"/>
+      <c r="H8" s="29" t="n"/>
+      <c r="I8" s="30" t="n"/>
     </row>
     <row r="9" ht="14.5" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
@@ -967,37 +923,37 @@
           <t>Data de Calibração:</t>
         </is>
       </c>
-      <c r="C9" s="35" t="inlineStr">
-        <is>
-          <t>29/01/2026</t>
-        </is>
-      </c>
-      <c r="D9" s="28" t="n"/>
+      <c r="C9" s="43" t="inlineStr">
+        <is>
+          <t>10/12/2024</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="n"/>
       <c r="E9" s="17" t="inlineStr">
         <is>
           <t>Empresa Certificadora:</t>
         </is>
       </c>
-      <c r="F9" s="26" t="inlineStr">
+      <c r="F9" s="28" t="inlineStr">
         <is>
           <t>ODS Metering Systems</t>
         </is>
       </c>
-      <c r="G9" s="27" t="n"/>
-      <c r="H9" s="27" t="n"/>
-      <c r="I9" s="28" t="n"/>
+      <c r="G9" s="29" t="n"/>
+      <c r="H9" s="29" t="n"/>
+      <c r="I9" s="30" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1"/>
     <row r="12" ht="12.75" customHeight="1">
-      <c r="B12" s="30" t="inlineStr">
+      <c r="B12" s="45" t="inlineStr">
         <is>
           <t>1.1 Descrição dos itens avaliados</t>
         </is>
       </c>
-      <c r="C12" s="27" t="n"/>
-      <c r="D12" s="27" t="n"/>
-      <c r="E12" s="27" t="n"/>
-      <c r="F12" s="28" t="n"/>
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="29" t="n"/>
+      <c r="E12" s="29" t="n"/>
+      <c r="F12" s="30" t="n"/>
       <c r="G12" s="5" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -1015,15 +971,15 @@
       </c>
     </row>
     <row r="13" ht="14.5" customHeight="1">
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="31" t="inlineStr">
         <is>
           <t>a) Identificação única do certificado (Número do Certificado de Calibração).</t>
         </is>
       </c>
-      <c r="C13" s="27" t="n"/>
-      <c r="D13" s="27" t="n"/>
-      <c r="E13" s="27" t="n"/>
-      <c r="F13" s="28" t="n"/>
+      <c r="C13" s="29" t="n"/>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="29" t="n"/>
+      <c r="F13" s="30" t="n"/>
       <c r="G13" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1033,15 +989,15 @@
       <c r="I13" s="23" t="n"/>
     </row>
     <row r="14" ht="14.5" customHeight="1">
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="31" t="inlineStr">
         <is>
           <t>b) Razão social e endereço do Laboratório/Empresa responsável.</t>
         </is>
       </c>
-      <c r="C14" s="27" t="n"/>
-      <c r="D14" s="27" t="n"/>
-      <c r="E14" s="27" t="n"/>
-      <c r="F14" s="28" t="n"/>
+      <c r="C14" s="29" t="n"/>
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="29" t="n"/>
+      <c r="F14" s="30" t="n"/>
       <c r="G14" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1051,15 +1007,15 @@
       <c r="I14" s="23" t="n"/>
     </row>
     <row r="15" ht="14.5" customHeight="1">
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="31" t="inlineStr">
         <is>
           <t>c) Presença do logotipo da RBC (quando aplicável a instrumentos associados a sistemas de medição fiscal, apropriação, custódia ou flare).</t>
         </is>
       </c>
-      <c r="C15" s="27" t="n"/>
-      <c r="D15" s="27" t="n"/>
-      <c r="E15" s="27" t="n"/>
-      <c r="F15" s="28" t="n"/>
+      <c r="C15" s="29" t="n"/>
+      <c r="D15" s="29" t="n"/>
+      <c r="E15" s="29" t="n"/>
+      <c r="F15" s="30" t="n"/>
       <c r="G15" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1069,15 +1025,15 @@
       <c r="I15" s="23" t="n"/>
     </row>
     <row r="16" ht="14.5" customHeight="1">
-      <c r="B16" s="29" t="inlineStr">
+      <c r="B16" s="31" t="inlineStr">
         <is>
           <t>d) Identificação do cliente (nome e endereço).</t>
         </is>
       </c>
-      <c r="C16" s="27" t="n"/>
-      <c r="D16" s="27" t="n"/>
-      <c r="E16" s="27" t="n"/>
-      <c r="F16" s="28" t="n"/>
+      <c r="C16" s="29" t="n"/>
+      <c r="D16" s="29" t="n"/>
+      <c r="E16" s="29" t="n"/>
+      <c r="F16" s="30" t="n"/>
       <c r="G16" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1087,15 +1043,15 @@
       <c r="I16" s="23" t="n"/>
     </row>
     <row r="17" ht="14.5" customHeight="1">
-      <c r="B17" s="29" t="inlineStr">
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>e) Indicação do número de páginas e total de páginas do documento.</t>
         </is>
       </c>
-      <c r="C17" s="27" t="n"/>
-      <c r="D17" s="27" t="n"/>
-      <c r="E17" s="27" t="n"/>
-      <c r="F17" s="28" t="n"/>
+      <c r="C17" s="29" t="n"/>
+      <c r="D17" s="29" t="n"/>
+      <c r="E17" s="29" t="n"/>
+      <c r="F17" s="30" t="n"/>
       <c r="G17" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1105,15 +1061,15 @@
       <c r="I17" s="23" t="n"/>
     </row>
     <row r="18" ht="14.5" customHeight="1">
-      <c r="B18" s="29" t="inlineStr">
+      <c r="B18" s="31" t="inlineStr">
         <is>
           <t>f) Identificação do método ou procedimento de calibração utilizado.</t>
         </is>
       </c>
-      <c r="C18" s="27" t="n"/>
-      <c r="D18" s="27" t="n"/>
-      <c r="E18" s="27" t="n"/>
-      <c r="F18" s="28" t="n"/>
+      <c r="C18" s="29" t="n"/>
+      <c r="D18" s="29" t="n"/>
+      <c r="E18" s="29" t="n"/>
+      <c r="F18" s="30" t="n"/>
       <c r="G18" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1123,15 +1079,15 @@
       <c r="I18" s="23" t="n"/>
     </row>
     <row r="19" ht="14.5" customHeight="1">
-      <c r="B19" s="29" t="inlineStr">
+      <c r="B19" s="31" t="inlineStr">
         <is>
           <t>g) Registro das condições ambientais durante a calibração.</t>
         </is>
       </c>
-      <c r="C19" s="27" t="n"/>
-      <c r="D19" s="27" t="n"/>
-      <c r="E19" s="27" t="n"/>
-      <c r="F19" s="28" t="n"/>
+      <c r="C19" s="29" t="n"/>
+      <c r="D19" s="29" t="n"/>
+      <c r="E19" s="29" t="n"/>
+      <c r="F19" s="30" t="n"/>
       <c r="G19" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1141,15 +1097,15 @@
       <c r="I19" s="23" t="n"/>
     </row>
     <row r="20" ht="14.5" customHeight="1">
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B20" s="31" t="inlineStr">
         <is>
           <t>h) Descrição e identificação do item calibrado (ex.: nome, fabricante, tipo, modelo, número de série, entre outros).</t>
         </is>
       </c>
-      <c r="C20" s="27" t="n"/>
-      <c r="D20" s="27" t="n"/>
-      <c r="E20" s="27" t="n"/>
-      <c r="F20" s="28" t="n"/>
+      <c r="C20" s="29" t="n"/>
+      <c r="D20" s="29" t="n"/>
+      <c r="E20" s="29" t="n"/>
+      <c r="F20" s="30" t="n"/>
       <c r="G20" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1159,15 +1115,15 @@
       <c r="I20" s="23" t="n"/>
     </row>
     <row r="21" ht="14.5" customHeight="1">
-      <c r="B21" s="29" t="inlineStr">
+      <c r="B21" s="31" t="inlineStr">
         <is>
           <t>i) Registro da data de recebimento do(s) item(ns) de calibração, quando aplicável.</t>
         </is>
       </c>
-      <c r="C21" s="27" t="n"/>
-      <c r="D21" s="27" t="n"/>
-      <c r="E21" s="27" t="n"/>
-      <c r="F21" s="28" t="n"/>
+      <c r="C21" s="29" t="n"/>
+      <c r="D21" s="29" t="n"/>
+      <c r="E21" s="29" t="n"/>
+      <c r="F21" s="30" t="n"/>
       <c r="G21" s="23" t="n"/>
       <c r="H21" s="23" t="n"/>
       <c r="I21" s="23" t="inlineStr">
@@ -1177,15 +1133,15 @@
       </c>
     </row>
     <row r="22" ht="14.5" customHeight="1">
-      <c r="B22" s="29" t="inlineStr">
+      <c r="B22" s="31" t="inlineStr">
         <is>
           <t>j) Indicação da data de realização da calibração.</t>
         </is>
       </c>
-      <c r="C22" s="27" t="n"/>
-      <c r="D22" s="27" t="n"/>
-      <c r="E22" s="27" t="n"/>
-      <c r="F22" s="28" t="n"/>
+      <c r="C22" s="29" t="n"/>
+      <c r="D22" s="29" t="n"/>
+      <c r="E22" s="29" t="n"/>
+      <c r="F22" s="30" t="n"/>
       <c r="G22" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1195,15 +1151,15 @@
       <c r="I22" s="23" t="n"/>
     </row>
     <row r="23" ht="14.5" customHeight="1">
-      <c r="B23" s="29" t="inlineStr">
+      <c r="B23" s="31" t="inlineStr">
         <is>
           <t>k) Apresentação dos resultados da calibração nas unidades de medida do Sistema Internacional (SI), quando aplicável.</t>
         </is>
       </c>
-      <c r="C23" s="27" t="n"/>
-      <c r="D23" s="27" t="n"/>
-      <c r="E23" s="27" t="n"/>
-      <c r="F23" s="28" t="n"/>
+      <c r="C23" s="29" t="n"/>
+      <c r="D23" s="29" t="n"/>
+      <c r="E23" s="29" t="n"/>
+      <c r="F23" s="30" t="n"/>
       <c r="G23" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1213,15 +1169,15 @@
       <c r="I23" s="23" t="n"/>
     </row>
     <row r="24" ht="14.5" customHeight="1">
-      <c r="B24" s="29" t="inlineStr">
+      <c r="B24" s="31" t="inlineStr">
         <is>
           <t>l) Evidências da rastreabilidade metrológica das medições (informações sobre os padrões utilizados).</t>
         </is>
       </c>
-      <c r="C24" s="27" t="n"/>
-      <c r="D24" s="27" t="n"/>
-      <c r="E24" s="27" t="n"/>
-      <c r="F24" s="28" t="n"/>
+      <c r="C24" s="29" t="n"/>
+      <c r="D24" s="29" t="n"/>
+      <c r="E24" s="29" t="n"/>
+      <c r="F24" s="30" t="n"/>
       <c r="G24" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1231,15 +1187,15 @@
       <c r="I24" s="23" t="n"/>
     </row>
     <row r="25" ht="24.75" customHeight="1">
-      <c r="B25" s="29" t="inlineStr">
+      <c r="B25" s="31" t="inlineStr">
         <is>
           <t>m) Identificação das pessoas autorizadas para emissão do certificado, incluindo nome(s), função(ões) e assinatura(s) ou identificação equivalente.</t>
         </is>
       </c>
-      <c r="C25" s="27" t="n"/>
-      <c r="D25" s="27" t="n"/>
-      <c r="E25" s="27" t="n"/>
-      <c r="F25" s="28" t="n"/>
+      <c r="C25" s="29" t="n"/>
+      <c r="D25" s="29" t="n"/>
+      <c r="E25" s="29" t="n"/>
+      <c r="F25" s="30" t="n"/>
       <c r="G25" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1249,15 +1205,15 @@
       <c r="I25" s="23" t="n"/>
     </row>
     <row r="26" ht="14.5" customHeight="1">
-      <c r="B26" s="29" t="inlineStr">
+      <c r="B26" s="31" t="inlineStr">
         <is>
           <t>n) Declaração de que os resultados e as incertezas apresentados referem-se exclusivamente aos itens calibrados e/ou inspecionados.</t>
         </is>
       </c>
-      <c r="C26" s="27" t="n"/>
-      <c r="D26" s="27" t="n"/>
-      <c r="E26" s="27" t="n"/>
-      <c r="F26" s="28" t="n"/>
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="29" t="n"/>
+      <c r="F26" s="30" t="n"/>
       <c r="G26" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1267,15 +1223,15 @@
       <c r="I26" s="23" t="n"/>
     </row>
     <row r="27" ht="14.5" customHeight="1">
-      <c r="B27" s="29" t="inlineStr">
+      <c r="B27" s="31" t="inlineStr">
         <is>
           <t>o) Indicação do nível de confiança e do fator de abrangência adotado.</t>
         </is>
       </c>
-      <c r="C27" s="27" t="n"/>
-      <c r="D27" s="27" t="n"/>
-      <c r="E27" s="27" t="n"/>
-      <c r="F27" s="28" t="n"/>
+      <c r="C27" s="29" t="n"/>
+      <c r="D27" s="29" t="n"/>
+      <c r="E27" s="29" t="n"/>
+      <c r="F27" s="30" t="n"/>
       <c r="G27" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1285,15 +1241,15 @@
       <c r="I27" s="23" t="n"/>
     </row>
     <row r="28" ht="14.5" customHeight="1">
-      <c r="B28" s="29" t="inlineStr">
+      <c r="B28" s="31" t="inlineStr">
         <is>
           <t>p) Verificação se a calibração foi realizada de acordo com a faixa solicitada pelo cliente.</t>
         </is>
       </c>
-      <c r="C28" s="27" t="n"/>
-      <c r="D28" s="27" t="n"/>
-      <c r="E28" s="27" t="n"/>
-      <c r="F28" s="28" t="n"/>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="29" t="n"/>
+      <c r="F28" s="30" t="n"/>
       <c r="G28" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1303,15 +1259,15 @@
       <c r="I28" s="23" t="n"/>
     </row>
     <row r="29" ht="24.75" customHeight="1">
-      <c r="B29" s="29" t="inlineStr">
+      <c r="B29" s="31" t="inlineStr">
         <is>
           <t>q) Confirmação de que os erros máximos de medição (erro sistemático remanescente somado à incerteza) são inferiores ao erro máximo admissível para o equipamento avaliado.</t>
         </is>
       </c>
-      <c r="C29" s="27" t="n"/>
-      <c r="D29" s="27" t="n"/>
-      <c r="E29" s="27" t="n"/>
-      <c r="F29" s="28" t="n"/>
+      <c r="C29" s="29" t="n"/>
+      <c r="D29" s="29" t="n"/>
+      <c r="E29" s="29" t="n"/>
+      <c r="F29" s="30" t="n"/>
       <c r="G29" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1321,15 +1277,15 @@
       <c r="I29" s="23" t="n"/>
     </row>
     <row r="30" ht="25.5" customHeight="1">
-      <c r="B30" s="29" t="inlineStr">
+      <c r="B30" s="31" t="inlineStr">
         <is>
           <t>r)  O instrumento está aprovado para uso no ponto de medição ao qual se destina, conforme os critérios de aceitação definidos pelo cliente ?</t>
         </is>
       </c>
-      <c r="C30" s="27" t="n"/>
-      <c r="D30" s="27" t="n"/>
-      <c r="E30" s="27" t="n"/>
-      <c r="F30" s="28" t="n"/>
+      <c r="C30" s="29" t="n"/>
+      <c r="D30" s="29" t="n"/>
+      <c r="E30" s="29" t="n"/>
+      <c r="F30" s="30" t="n"/>
       <c r="G30" s="23" t="inlineStr">
         <is>
           <t>X</t>
@@ -1339,15 +1295,15 @@
       <c r="I30" s="23" t="n"/>
     </row>
     <row r="31" ht="25.5" customHeight="1">
-      <c r="B31" s="29" t="inlineStr">
+      <c r="B31" s="31" t="inlineStr">
         <is>
           <t>s) Quando houver ajuste no equipamento, apresentação dos resultados de calibração nas condições “como encontrado” (as found) e “como deixado” (as left).</t>
         </is>
       </c>
-      <c r="C31" s="27" t="n"/>
-      <c r="D31" s="27" t="n"/>
-      <c r="E31" s="27" t="n"/>
-      <c r="F31" s="28" t="n"/>
+      <c r="C31" s="29" t="n"/>
+      <c r="D31" s="29" t="n"/>
+      <c r="E31" s="29" t="n"/>
+      <c r="F31" s="30" t="n"/>
       <c r="G31" s="23" t="n"/>
       <c r="H31" s="23" t="n"/>
       <c r="I31" s="23" t="inlineStr">
@@ -1357,53 +1313,53 @@
       </c>
     </row>
     <row r="32" ht="27" customHeight="1">
-      <c r="B32" s="36" t="inlineStr">
+      <c r="B32" s="33" t="inlineStr">
         <is>
           <t>1.2 Recomenda-se que o relatório de análise contenha identificação adequada e informações claras sobre o emitente.
 O relatório apresentado está em conformidade com essa recomendação?</t>
         </is>
       </c>
-      <c r="C32" s="27" t="n"/>
-      <c r="D32" s="27" t="n"/>
-      <c r="E32" s="27" t="n"/>
-      <c r="F32" s="27" t="n"/>
-      <c r="G32" s="27" t="n"/>
-      <c r="H32" s="27" t="n"/>
-      <c r="I32" s="28" t="n"/>
+      <c r="C32" s="29" t="n"/>
+      <c r="D32" s="29" t="n"/>
+      <c r="E32" s="29" t="n"/>
+      <c r="F32" s="29" t="n"/>
+      <c r="G32" s="29" t="n"/>
+      <c r="H32" s="29" t="n"/>
+      <c r="I32" s="30" t="n"/>
     </row>
     <row r="33" ht="66.75" customHeight="1">
-      <c r="B33" s="42" t="inlineStr">
+      <c r="B33" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">( X )   Sim      (   ) Não
 OBSERVAÇÕES:
 </t>
         </is>
       </c>
-      <c r="C33" s="27" t="n"/>
-      <c r="D33" s="27" t="n"/>
-      <c r="E33" s="27" t="n"/>
-      <c r="F33" s="27" t="n"/>
-      <c r="G33" s="27" t="n"/>
-      <c r="H33" s="27" t="n"/>
-      <c r="I33" s="28" t="n"/>
+      <c r="C33" s="29" t="n"/>
+      <c r="D33" s="29" t="n"/>
+      <c r="E33" s="29" t="n"/>
+      <c r="F33" s="29" t="n"/>
+      <c r="G33" s="29" t="n"/>
+      <c r="H33" s="29" t="n"/>
+      <c r="I33" s="30" t="n"/>
     </row>
     <row r="34" ht="45" customHeight="1">
-      <c r="B34" s="38" t="inlineStr">
+      <c r="B34" s="34" t="inlineStr">
         <is>
           <t>1.3 Existe alguma informação no documento analisado que necessite complementação, correção ou esclarecimento para melhor compreensão do dispositivo
 (ex.: faixa de calibração no computador de vazão)?</t>
         </is>
       </c>
-      <c r="C34" s="27" t="n"/>
-      <c r="D34" s="27" t="n"/>
-      <c r="E34" s="27" t="n"/>
-      <c r="F34" s="27" t="n"/>
-      <c r="G34" s="27" t="n"/>
-      <c r="H34" s="27" t="n"/>
-      <c r="I34" s="28" t="n"/>
+      <c r="C34" s="29" t="n"/>
+      <c r="D34" s="29" t="n"/>
+      <c r="E34" s="29" t="n"/>
+      <c r="F34" s="29" t="n"/>
+      <c r="G34" s="29" t="n"/>
+      <c r="H34" s="29" t="n"/>
+      <c r="I34" s="30" t="n"/>
     </row>
     <row r="35" ht="77.25" customHeight="1">
-      <c r="B35" s="45" t="inlineStr">
+      <c r="B35" s="44" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -1413,72 +1369,72 @@
           </r>
         </is>
       </c>
-      <c r="C35" s="27" t="n"/>
-      <c r="D35" s="27" t="n"/>
-      <c r="E35" s="27" t="n"/>
-      <c r="F35" s="27" t="n"/>
-      <c r="G35" s="27" t="n"/>
-      <c r="H35" s="27" t="n"/>
-      <c r="I35" s="28" t="n"/>
+      <c r="C35" s="29" t="n"/>
+      <c r="D35" s="29" t="n"/>
+      <c r="E35" s="29" t="n"/>
+      <c r="F35" s="29" t="n"/>
+      <c r="G35" s="29" t="n"/>
+      <c r="H35" s="29" t="n"/>
+      <c r="I35" s="30" t="n"/>
     </row>
     <row r="36" ht="27.75" customHeight="1">
-      <c r="B36" s="37" t="inlineStr">
+      <c r="B36" s="32" t="inlineStr">
         <is>
           <t>1.4 Com base na data do último ensaio ou análise registrada, bem como no critério de periodicidade definido para sua execução, a periodicidade estabelecida foi atendida?</t>
         </is>
       </c>
-      <c r="C36" s="27" t="n"/>
-      <c r="D36" s="27" t="n"/>
-      <c r="E36" s="27" t="n"/>
-      <c r="F36" s="27" t="n"/>
-      <c r="G36" s="27" t="n"/>
-      <c r="H36" s="27" t="n"/>
-      <c r="I36" s="28" t="n"/>
+      <c r="C36" s="29" t="n"/>
+      <c r="D36" s="29" t="n"/>
+      <c r="E36" s="29" t="n"/>
+      <c r="F36" s="29" t="n"/>
+      <c r="G36" s="29" t="n"/>
+      <c r="H36" s="29" t="n"/>
+      <c r="I36" s="30" t="n"/>
     </row>
     <row r="37" ht="63.75" customHeight="1">
-      <c r="B37" s="39" t="inlineStr">
+      <c r="B37" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">(   X   )  Sim       (      ) Não
 OBSERVAÇÕES: </t>
         </is>
       </c>
-      <c r="C37" s="27" t="n"/>
-      <c r="D37" s="27" t="n"/>
-      <c r="E37" s="27" t="n"/>
-      <c r="F37" s="27" t="n"/>
-      <c r="G37" s="27" t="n"/>
-      <c r="H37" s="27" t="n"/>
-      <c r="I37" s="28" t="n"/>
+      <c r="C37" s="29" t="n"/>
+      <c r="D37" s="29" t="n"/>
+      <c r="E37" s="29" t="n"/>
+      <c r="F37" s="29" t="n"/>
+      <c r="G37" s="29" t="n"/>
+      <c r="H37" s="29" t="n"/>
+      <c r="I37" s="30" t="n"/>
     </row>
     <row r="38" ht="28.5" customHeight="1">
-      <c r="B38" s="37" t="inlineStr">
+      <c r="B38" s="32" t="inlineStr">
         <is>
           <t>1.5 Conclusão da análise crítica do relatório de calibração
 O certificado está em conformidade com os requisitos do cliente e da RTM?</t>
         </is>
       </c>
-      <c r="C38" s="27" t="n"/>
-      <c r="D38" s="27" t="n"/>
-      <c r="E38" s="27" t="n"/>
-      <c r="F38" s="27" t="n"/>
-      <c r="G38" s="27" t="n"/>
-      <c r="H38" s="27" t="n"/>
-      <c r="I38" s="28" t="n"/>
+      <c r="C38" s="29" t="n"/>
+      <c r="D38" s="29" t="n"/>
+      <c r="E38" s="29" t="n"/>
+      <c r="F38" s="29" t="n"/>
+      <c r="G38" s="29" t="n"/>
+      <c r="H38" s="29" t="n"/>
+      <c r="I38" s="30" t="n"/>
     </row>
     <row r="39" ht="64.5" customHeight="1">
-      <c r="B39" s="31" t="inlineStr">
+      <c r="B39" s="39" t="inlineStr">
         <is>
           <t>(   X   )  Sim       (      ) Não*
 *Caso a resposta seja “Não”, justifique:</t>
         </is>
       </c>
-      <c r="C39" s="32" t="n"/>
-      <c r="D39" s="32" t="n"/>
-      <c r="E39" s="32" t="n"/>
-      <c r="F39" s="32" t="n"/>
-      <c r="G39" s="32" t="n"/>
-      <c r="H39" s="32" t="n"/>
-      <c r="I39" s="33" t="n"/>
+      <c r="C39" s="40" t="n"/>
+      <c r="D39" s="40" t="n"/>
+      <c r="E39" s="40" t="n"/>
+      <c r="F39" s="40" t="n"/>
+      <c r="G39" s="40" t="n"/>
+      <c r="H39" s="40" t="n"/>
+      <c r="I39" s="41" t="n"/>
     </row>
     <row r="40" ht="33" customHeight="1">
       <c r="B40" s="6" t="n"/>
@@ -1493,7 +1449,7 @@
       <c r="G40" s="18" t="n"/>
       <c r="H40" s="19" t="inlineStr">
         <is>
-          <t>02/02/2026</t>
+          <t>16/12/2024</t>
         </is>
       </c>
       <c r="I40" s="20" t="n"/>
@@ -1501,12 +1457,12 @@
     <row r="41" ht="36" customHeight="1">
       <c r="B41" s="8" t="n"/>
       <c r="C41" s="9" t="n"/>
-      <c r="D41" s="34" t="inlineStr">
+      <c r="D41" s="42" t="inlineStr">
         <is>
           <t>Responsável pela análise</t>
         </is>
       </c>
-      <c r="E41" s="27" t="n"/>
+      <c r="E41" s="29" t="n"/>
       <c r="F41" s="9" t="n"/>
       <c r="G41" s="9" t="n"/>
       <c r="H41" s="9" t="n"/>

</xml_diff>

<commit_message>
ajuste solicitação de sobrescrita de AC ao usuário
</commit_message>
<xml_diff>
--- a/TemplateAC_YINSON.xlsx
+++ b/TemplateAC_YINSON.xlsx
@@ -824,7 +824,7 @@
       <c r="B2" s="13" t="n"/>
       <c r="C2" s="25" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Sensores de Temperatura</t>
+          <t>Análise Crítica de Calibração dos Transmissores de Pressão</t>
         </is>
       </c>
       <c r="D2" s="21" t="n"/>
@@ -884,7 +884,7 @@
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>27TE2502</t>
+          <t>27FT2502B</t>
         </is>
       </c>
       <c r="G7" s="27" t="n"/>
@@ -910,7 +910,7 @@
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>26-ODS-95 - TEM - 038</t>
+          <t>26-ODS-95 - PRE - 029</t>
         </is>
       </c>
       <c r="G8" s="27" t="n"/>
@@ -1481,9 +1481,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="C9:D9"/>
-    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B32:I32"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>

</xml_diff>

<commit_message>
geração xml cromatografia sgs
</commit_message>
<xml_diff>
--- a/TemplateAC_YINSON.xlsx
+++ b/TemplateAC_YINSON.xlsx
@@ -910,7 +910,7 @@
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>24‐ODS‐95 ‐ PRE ‐ 974</t>
+          <t>24‐ODS‐95‐PRE‐974</t>
         </is>
       </c>
       <c r="G8" s="27" t="n"/>
@@ -1481,9 +1481,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="C9:D9"/>
     <mergeCell ref="D41:E41"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="C9:D9"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B29:F29"/>

</xml_diff>